<commit_message>
feat: implementasi Bagian C, custom a8 options, dan edit detail hasil lengkap
</commit_message>
<xml_diff>
--- a/template-instrumen-baru.xlsx
+++ b/template-instrumen-baru.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus VivoBook\Documents\LOCALHOST\interview-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2850A0A6-4082-4AE5-BF38-369D3D2D0ACC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB60C644-DCF6-4133-8514-912E6F40A363}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="13008" windowHeight="11256" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="21336" windowHeight="11376" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="170">
   <si>
     <t>ID</t>
   </si>
@@ -524,6 +524,27 @@
   </si>
   <si>
     <t>b42</t>
+  </si>
+  <si>
+    <t>c1</t>
+  </si>
+  <si>
+    <t>C. KOMITMEN PROGRAM ETOS ID</t>
+  </si>
+  <si>
+    <t>Kesiapan Mengikuti Program &amp; Peraturan</t>
+  </si>
+  <si>
+    <t>Jika Anda diterima sebagai penerima beasiswa Etos ID, apakah Anda siap mengikuti seluruh program dan peraturan yang berlaku—seperti tidak merokok, tidak berpacaran, tinggal di asrama, target hafalan Qur'an, kegiatan pembinaan rutin, dan pelaporan perkembangan akademik secara berkala?</t>
+  </si>
+  <si>
+    <t>Memiliki keyakinan dan semangat penuh untuk mengikuti seluruh program &amp; peraturan Etos ID tanpa keberatan.</t>
+  </si>
+  <si>
+    <t>Belum sepenuhnya yakin/masih ragu dapat mengikuti seluruh peraturan dan program dengan konsisten.</t>
+  </si>
+  <si>
+    <t>c2</t>
   </si>
 </sst>
 </file>
@@ -912,7 +933,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr defaultRowHeight="141.6" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.5" style="1" bestFit="1" customWidth="1"/>
@@ -2098,6 +2119,52 @@
         <v>70</v>
       </c>
     </row>
+    <row r="52" spans="1:7" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="F52" s="2">
+        <v>1</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" ht="141.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="F53" s="2">
+        <v>0</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>